<commit_message>
Fix Argentina results and pending changes research
</commit_message>
<xml_diff>
--- a/docs/research/argentina/argentina-research-v3.0.xlsx
+++ b/docs/research/argentina/argentina-research-v3.0.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="1" r:id="Rdd87c7f3b89749fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Страна" sheetId="2" r:id="R926fb735301f4523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Маршруты" sheetId="3" r:id="Rcbf094e757444e0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Доход" sheetId="4" r:id="R439dca2b22174cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Семья" sheetId="5" r:id="Rda2bcbfab85c4c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Работа" sheetId="6" r:id="R6b7efa56e9ea40f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_ПМЖ_Гражданство" sheetId="7" r:id="Ref244b4e00544373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Города" sheetId="8" r:id="R9a9d4c63a3f74524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Школы" sheetId="9" r:id="R2bc363d9e4264d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Животные" sheetId="10" r:id="Rae2c93465fa245c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_ЛГБТ" sheetId="11" r:id="R455a6a0e37c84730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Источники" sheetId="12" r:id="Rfc31ba2d2f934726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Словарь" sheetId="13" r:id="R6663347eb5974fc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Полнота" sheetId="14" r:id="Rb5542bb9c0dd4bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Открытые_вопросы" sheetId="15" r:id="Rb96f2158436f49c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Исключено" sheetId="16" r:id="R10d4b13013ff4e8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_QA" sheetId="17" r:id="Rc8605d18354141e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="1" r:id="R96085617e6074ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Страна" sheetId="2" r:id="R68b748c5a43b4aa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Маршруты" sheetId="3" r:id="Rc6da28737ff74cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Доход" sheetId="4" r:id="R11e010f3be27494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Семья" sheetId="5" r:id="R7b72e4584dc54fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Работа" sheetId="6" r:id="Rc0744663a7954d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_ПМЖ_Гражданство" sheetId="7" r:id="Rae8ca75966774e5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Города" sheetId="8" r:id="R2db93187582f484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Школы" sheetId="9" r:id="Re5a3643a1e494ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Животные" sheetId="10" r:id="Rab568729815b4239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_ЛГБТ" sheetId="11" r:id="R2cfb2fab38d14a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Источники" sheetId="12" r:id="Rfe674510870641ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Словарь" sheetId="13" r:id="R1def93224cbd4282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Полнота" sheetId="14" r:id="R04f49bb70b064bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Открытые_вопросы" sheetId="15" r:id="R4c1a806dcef846cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Исключено" sheetId="16" r:id="R1dd91c90e01c4293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_QA" sheetId="17" r:id="R8cbd39bc57bc49e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -158,6 +158,7 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -320,7 +321,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Аргентина — исследование v3.0</x:v>
+        <x:v>Аргентина — исследование v3.0 (РФ-only MVP)</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -367,7 +368,7 @@
         <x:v>Публикуемые маршруты</x:v>
       </x:c>
       <x:c r="B7" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -383,7 +384,7 @@
         <x:v>Статус</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>Готова к подключению для 8 маршрутов; инвесторская резиденция и гражданство за инвестицию скрыты до публикации критериев.</x:v>
+        <x:v>Готова к подключению для 6 маршрутов, которые можно оценить по универсальной анкете гражданина РФ; инвесторская резиденция скрыта до публикации критериев.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -484,6 +485,7 @@
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -505,6 +507,9 @@
       <x:c r="F1" s="18" t="str">
         <x:v>Международная защита</x:v>
       </x:c>
+      <x:c r="G1" s="10" t="str">
+        <x:v>Что меняется (только будущие правила)</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="30" t="str">
@@ -525,6 +530,15 @@
       <x:c r="F2" s="30" t="str">
         <x:v>Международная защита, то есть убежище, возможна при обоснованном страхе преследования, включая преследование из-за принадлежности к определённой социальной группе. Для ЛГБТ-заявителя это может охватывать преследование из-за сексуальной ориентации или гендерной идентичности. Это отдельная процедура, а не обычный ВНЖ.</x:v>
       </x:c>
+      <x:c r="G2" s="10" t="str">
+        <x:v>Нет подтверждённых будущих изменений</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="G3" s="10"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="G4" s="10"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -937,7 +951,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="30" t="str">
-        <x:v>AR_SRC_MERCOSUR</x:v>
+        <x:v>AR_SRC_PR</x:v>
       </x:c>
       <x:c r="B16" s="30" t="str">
         <x:v>OFFICIAL</x:v>
@@ -946,13 +960,13 @@
         <x:v>Национальное управление миграции Аргентины</x:v>
       </x:c>
       <x:c r="D16" s="30" t="str">
-        <x:v>Временная резиденция по гражданству страны МЕРКОСУР</x:v>
+        <x:v>Частые вопросы о постоянной резиденции</x:v>
       </x:c>
       <x:c r="E16" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/servicio/obtener-una-residencia-temporaria-por-nacionalidad-mercosur</x:v>
+        <x:v>https://www.argentina.gob.ar/migraciones/preguntas-frecuentes-residencias</x:v>
       </x:c>
       <x:c r="F16" s="30" t="str">
-        <x:v>2 года; доступна при подходящем втором гражданстве.</x:v>
+        <x:v>Для гражданина РФ ПМЖ после 3 лет временной резиденции при присутствии в Аргентине более 50% срока.</x:v>
       </x:c>
       <x:c r="G16" s="30" t="str">
         <x:v>2026-07-24</x:v>
@@ -963,22 +977,22 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="26" t="str">
-        <x:v>AR_SRC_PR</x:v>
+        <x:v>AR_SRC_MIGRATION_LAW</x:v>
       </x:c>
       <x:c r="B17" s="26" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C17" s="26" t="str">
-        <x:v>Национальное управление миграции Аргентины</x:v>
+        <x:v>Законодательство Аргентины</x:v>
       </x:c>
       <x:c r="D17" s="26" t="str">
-        <x:v>Частые вопросы о постоянной резиденции</x:v>
+        <x:v>Закон о миграции № 25.871, актуальная редакция</x:v>
       </x:c>
       <x:c r="E17" s="26" t="str">
-        <x:v>https://www.argentina.gob.ar/migraciones/preguntas-frecuentes-residencias</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/ley-25871-92016/actualizacion</x:v>
       </x:c>
       <x:c r="F17" s="26" t="str">
-        <x:v>ПМЖ после 2 лет временной резиденции для МЕРКОСУР и 3 лет для остальных; присутствие в Аргентине более 50% срока.</x:v>
+        <x:v>Категории резиденций, инвестор, права временных резидентов на работу и бизнес, признание зарегистрированного фактического партнёрства.</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
         <x:v>2026-07-24</x:v>
@@ -989,7 +1003,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
-        <x:v>AR_SRC_MIGRATION_LAW</x:v>
+        <x:v>AR_SRC_CITIZENSHIP</x:v>
       </x:c>
       <x:c r="B18" s="30" t="str">
         <x:v>OFFICIAL</x:v>
@@ -998,13 +1012,13 @@
         <x:v>Законодательство Аргентины</x:v>
       </x:c>
       <x:c r="D18" s="30" t="str">
-        <x:v>Закон о миграции № 25.871, актуальная редакция</x:v>
+        <x:v>Закон о гражданстве № 346, актуальная редакция</x:v>
       </x:c>
       <x:c r="E18" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/ley-25871-92016/actualizacion</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/ley-346-48854/actualizacion</x:v>
       </x:c>
       <x:c r="F18" s="30" t="str">
-        <x:v>Категории резиденций, инвестор, права временных резидентов на работу и бизнес, признание зарегистрированного фактического партнёрства.</x:v>
+        <x:v>2 года непрерывного законного проживания без единого выезда; отдельная норма о гражданстве за значимую инвестицию.</x:v>
       </x:c>
       <x:c r="G18" s="30" t="str">
         <x:v>2026-07-24</x:v>
@@ -1015,22 +1029,22 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="26" t="str">
-        <x:v>AR_SRC_CITIZENSHIP</x:v>
+        <x:v>AR_SRC_INVEST_CIT</x:v>
       </x:c>
       <x:c r="B19" s="26" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C19" s="26" t="str">
-        <x:v>Законодательство Аргентины</x:v>
+        <x:v>Правительство Аргентины</x:v>
       </x:c>
       <x:c r="D19" s="26" t="str">
-        <x:v>Закон о гражданстве № 346, актуальная редакция</x:v>
+        <x:v>Процедура гражданства за значимую инвестицию</x:v>
       </x:c>
       <x:c r="E19" s="26" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/ley-346-48854/actualizacion</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/decreto-524-2025-415710/texto</x:v>
       </x:c>
       <x:c r="F19" s="26" t="str">
-        <x:v>2 года непрерывного законного проживания без единого выезда; отдельная норма о гражданстве за значимую инвестицию.</x:v>
+        <x:v>Процедура создана, но критерии значимой инвестиции должен определить Минэкономики; универсальная сумма не опубликована.</x:v>
       </x:c>
       <x:c r="G19" s="26" t="str">
         <x:v>2026-07-24</x:v>
@@ -1041,22 +1055,22 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="30" t="str">
-        <x:v>AR_SRC_INVEST_CIT</x:v>
+        <x:v>AR_SRC_DUAL_RU</x:v>
       </x:c>
       <x:c r="B20" s="30" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C20" s="30" t="str">
-        <x:v>Правительство Аргентины</x:v>
+        <x:v>Президент России / Федеральный закон № 138-ФЗ</x:v>
       </x:c>
       <x:c r="D20" s="30" t="str">
-        <x:v>Процедура гражданства за значимую инвестицию</x:v>
+        <x:v>Сохранение гражданства РФ при приобретении иностранного гражданства</x:v>
       </x:c>
       <x:c r="E20" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/decreto-524-2025-415710/texto</x:v>
+        <x:v>https://www.kremlin.ru/acts/bank/49216/print</x:v>
       </x:c>
       <x:c r="F20" s="30" t="str">
-        <x:v>Процедура создана, но критерии значимой инвестиции должен определить Минэкономики; универсальная сумма не опубликована.</x:v>
+        <x:v>Приобретение иностранного гражданства не прекращает гражданство РФ; действует обязанность уведомления в предусмотренных законом случаях.</x:v>
       </x:c>
       <x:c r="G20" s="30" t="str">
         <x:v>2026-07-24</x:v>
@@ -1067,22 +1081,22 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="26" t="str">
-        <x:v>AR_SRC_DUAL_RU</x:v>
+        <x:v>AR_SRC_SCHOOL_ACCESS</x:v>
       </x:c>
       <x:c r="B21" s="26" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C21" s="26" t="str">
-        <x:v>Президент России / Федеральный закон № 138-ФЗ</x:v>
+        <x:v>Законодательство Аргентины</x:v>
       </x:c>
       <x:c r="D21" s="26" t="str">
-        <x:v>Сохранение гражданства РФ при приобретении иностранного гражданства</x:v>
+        <x:v>Закон об образовании — доступ детей мигрантов</x:v>
       </x:c>
       <x:c r="E21" s="26" t="str">
-        <x:v>https://www.kremlin.ru/acts/bank/49216/print</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/123542/actualizacion</x:v>
       </x:c>
       <x:c r="F21" s="26" t="str">
-        <x:v>Приобретение иностранного гражданства не прекращает гражданство РФ; действует обязанность уведомления в предусмотренных законом случаях.</x:v>
+        <x:v>Доступ к начальному и среднему образованию гарантирован детям мигрантов, даже без аргентинского удостоверения личности.</x:v>
       </x:c>
       <x:c r="G21" s="26" t="str">
         <x:v>2026-07-24</x:v>
@@ -1093,22 +1107,22 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="30" t="str">
-        <x:v>AR_SRC_SCHOOL_ACCESS</x:v>
+        <x:v>AR_SRC_PETS</x:v>
       </x:c>
       <x:c r="B22" s="30" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C22" s="30" t="str">
-        <x:v>Законодательство Аргентины</x:v>
+        <x:v>SENASA</x:v>
       </x:c>
       <x:c r="D22" s="30" t="str">
-        <x:v>Закон об образовании — доступ детей мигрантов</x:v>
+        <x:v>Ввоз собак и кошек</x:v>
       </x:c>
       <x:c r="E22" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/123542/actualizacion</x:v>
+        <x:v>https://www.argentina.gob.ar/senasa/informacion-al-viajero/ingresar-o-regresar-al-pais/ingresos-con-perros-yo-gatos</x:v>
       </x:c>
       <x:c r="F22" s="30" t="str">
-        <x:v>Доступ к начальному и среднему образованию гарантирован детям мигрантов, даже без аргентинского удостоверения личности.</x:v>
+        <x:v>Ввоз разрешён; предварительное разрешение для сопровождаемого животного и обычный карантин не требуются; национальный запрет пород не указан.</x:v>
       </x:c>
       <x:c r="G22" s="30" t="str">
         <x:v>2026-07-24</x:v>
@@ -1119,22 +1133,22 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="26" t="str">
-        <x:v>AR_SRC_PETS</x:v>
+        <x:v>AR_SRC_MARRIAGE</x:v>
       </x:c>
       <x:c r="B23" s="26" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C23" s="26" t="str">
-        <x:v>SENASA</x:v>
+        <x:v>Законодательство Аргентины</x:v>
       </x:c>
       <x:c r="D23" s="26" t="str">
-        <x:v>Ввоз собак и кошек</x:v>
+        <x:v>Закон о равном браке № 26.618</x:v>
       </x:c>
       <x:c r="E23" s="26" t="str">
-        <x:v>https://www.argentina.gob.ar/senasa/informacion-al-viajero/ingresar-o-regresar-al-pais/ingresos-con-perros-yo-gatos</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/169608/texto</x:v>
       </x:c>
       <x:c r="F23" s="26" t="str">
-        <x:v>Ввоз разрешён; предварительное разрешение для сопровождаемого животного и обычный карантин не требуются; национальный запрет пород не указан.</x:v>
+        <x:v>Однополый и разнополый брак имеют одинаковые требования и последствия.</x:v>
       </x:c>
       <x:c r="G23" s="26" t="str">
         <x:v>2026-07-24</x:v>
@@ -1145,22 +1159,22 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30" t="str">
-        <x:v>AR_SRC_MARRIAGE</x:v>
+        <x:v>AR_SRC_PARTNERSHIP</x:v>
       </x:c>
       <x:c r="B24" s="30" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C24" s="30" t="str">
-        <x:v>Законодательство Аргентины</x:v>
+        <x:v>Министерство юстиции Аргентины</x:v>
       </x:c>
       <x:c r="D24" s="30" t="str">
-        <x:v>Закон о равном браке № 26.618</x:v>
+        <x:v>Зарегистрированное фактическое партнёрство</x:v>
       </x:c>
       <x:c r="E24" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/169608/texto</x:v>
+        <x:v>https://www.argentina.gob.ar/justicia/derechofacil/leysimple/uniones-convivenciales</x:v>
       </x:c>
       <x:c r="F24" s="30" t="str">
-        <x:v>Однополый и разнополый брак имеют одинаковые требования и последствия.</x:v>
+        <x:v>Официально зарегистрированное совместное проживание пары без брака; доступно однополым и разнополым парам.</x:v>
       </x:c>
       <x:c r="G24" s="30" t="str">
         <x:v>2026-07-24</x:v>
@@ -1171,22 +1185,22 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="26" t="str">
-        <x:v>AR_SRC_PARTNERSHIP</x:v>
+        <x:v>AR_SRC_ASYLUM</x:v>
       </x:c>
       <x:c r="B25" s="26" t="str">
         <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C25" s="26" t="str">
-        <x:v>Министерство юстиции Аргентины</x:v>
+        <x:v>Законодательство Аргентины</x:v>
       </x:c>
       <x:c r="D25" s="26" t="str">
-        <x:v>Зарегистрированное фактическое партнёрство</x:v>
+        <x:v>Закон о признании и защите беженцев № 26.165</x:v>
       </x:c>
       <x:c r="E25" s="26" t="str">
-        <x:v>https://www.argentina.gob.ar/justicia/derechofacil/leysimple/uniones-convivenciales</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/ley-26165-122609/actualizacion</x:v>
       </x:c>
       <x:c r="F25" s="26" t="str">
-        <x:v>Официально зарегистрированное совместное проживание пары без брака; доступно однополым и разнополым парам.</x:v>
+        <x:v>Международная защита возможна при обоснованном страхе преследования, включая принадлежность к определённой социальной группе.</x:v>
       </x:c>
       <x:c r="G25" s="26" t="str">
         <x:v>2026-07-24</x:v>
@@ -1197,133 +1211,117 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="30" t="str">
-        <x:v>AR_SRC_ASYLUM</x:v>
+        <x:v>AR_SRC_CITY_COST</x:v>
       </x:c>
       <x:c r="B26" s="30" t="str">
-        <x:v>OFFICIAL</x:v>
+        <x:v>PRACTICAL</x:v>
       </x:c>
       <x:c r="C26" s="30" t="str">
-        <x:v>Законодательство Аргентины</x:v>
+        <x:v>CityCost</x:v>
       </x:c>
       <x:c r="D26" s="30" t="str">
-        <x:v>Закон о признании и защите беженцев № 26.165</x:v>
+        <x:v>Сравнимые оценки стоимости жизни в городах Аргентины</x:v>
       </x:c>
       <x:c r="E26" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/ley-26165-122609/actualizacion</x:v>
+        <x:v>https://citycost.org/argentina/</x:v>
       </x:c>
       <x:c r="F26" s="30" t="str">
-        <x:v>Международная защита возможна при обоснованном страхе преследования, включая принадлежность к определённой социальной группе.</x:v>
+        <x:v>Ориентировочные бюджеты с арендой по выбранным городам; вторичный источник.</x:v>
       </x:c>
       <x:c r="G26" s="30" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="H26" s="30" t="str">
-        <x:v>HIGH</x:v>
+        <x:v>MEDIUM</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="26" t="str">
-        <x:v>AR_SRC_CITY_COST</x:v>
+        <x:v>AR_SRC_CLIMATE</x:v>
       </x:c>
       <x:c r="B27" s="26" t="str">
-        <x:v>PRACTICAL</x:v>
+        <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C27" s="26" t="str">
-        <x:v>CityCost</x:v>
+        <x:v>Национальная метеорологическая служба Аргентины</x:v>
       </x:c>
       <x:c r="D27" s="26" t="str">
-        <x:v>Сравнимые оценки стоимости жизни в городах Аргентины</x:v>
+        <x:v>Климатические нормы 1991–2020</x:v>
       </x:c>
       <x:c r="E27" s="26" t="str">
-        <x:v>https://citycost.org/argentina/</x:v>
+        <x:v>https://repositorio.smn.gob.ar/handle/20.500.12160/2506</x:v>
       </x:c>
       <x:c r="F27" s="26" t="str">
-        <x:v>Ориентировочные бюджеты с арендой по выбранным городам; вторичный источник.</x:v>
+        <x:v>Официальные многолетние климатические нормы по метеостанциям.</x:v>
       </x:c>
       <x:c r="G27" s="26" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="H27" s="26" t="str">
-        <x:v>MEDIUM</x:v>
+        <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="30" t="str">
-        <x:v>AR_SRC_CLIMATE</x:v>
+        <x:v>AR_SRC_USHUAIA_SCHOOL</x:v>
       </x:c>
       <x:c r="B28" s="30" t="str">
-        <x:v>OFFICIAL</x:v>
+        <x:v>PRACTICAL</x:v>
       </x:c>
       <x:c r="C28" s="30" t="str">
-        <x:v>Национальная метеорологическая служба Аргентины</x:v>
+        <x:v>Colegio Nacional de Ushuaia</x:v>
       </x:c>
       <x:c r="D28" s="30" t="str">
-        <x:v>Климатические нормы 1991–2020</x:v>
+        <x:v>Школа в Ушуайе с международными экзаменами по английскому</x:v>
       </x:c>
       <x:c r="E28" s="30" t="str">
-        <x:v>https://repositorio.smn.gob.ar/handle/20.500.12160/2506</x:v>
+        <x:v>https://www.cnu.edu.ar/institucional</x:v>
       </x:c>
       <x:c r="F28" s="30" t="str">
-        <x:v>Официальные многолетние климатические нормы по метеостанциям.</x:v>
+        <x:v>Есть местная школа с международными экзаменами, но полноценная международная программа и цена не подтверждены.</x:v>
       </x:c>
       <x:c r="G28" s="30" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="H28" s="30" t="str">
-        <x:v>HIGH</x:v>
+        <x:v>MEDIUM</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="26" t="str">
-        <x:v>AR_SRC_USHUAIA_SCHOOL</x:v>
+        <x:v>AR_SRC_RENT_AMEND</x:v>
       </x:c>
       <x:c r="B29" s="26" t="str">
-        <x:v>PRACTICAL</x:v>
+        <x:v>OFFICIAL</x:v>
       </x:c>
       <x:c r="C29" s="26" t="str">
-        <x:v>Colegio Nacional de Ushuaia</x:v>
+        <x:v>Национальное управление миграции Аргентины</x:v>
       </x:c>
       <x:c r="D29" s="26" t="str">
-        <x:v>Школа в Ушуайе с международными экзаменами по английскому</x:v>
+        <x:v>Изменение финансового правила рантье и пенсионера 2023 года</x:v>
       </x:c>
       <x:c r="E29" s="26" t="str">
-        <x:v>https://www.cnu.edu.ar/institucional</x:v>
+        <x:v>https://www.argentina.gob.ar/normativa/nacional/disposici%C3%B3n-3446-2023-392424/texto</x:v>
       </x:c>
       <x:c r="F29" s="26" t="str">
-        <x:v>Есть местная школа с международными экзаменами, но полноценная международная программа и цена не подтверждены.</x:v>
+        <x:v>Действующая формулировка: минимум 5 официальных минимальных зарплат; прежняя фраза о сумме на каждого заявителя заменена.</x:v>
       </x:c>
       <x:c r="G29" s="26" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="H29" s="26" t="str">
-        <x:v>MEDIUM</x:v>
+        <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="30" t="str">
-        <x:v>AR_SRC_RENT_AMEND</x:v>
-      </x:c>
-      <x:c r="B30" s="30" t="str">
-        <x:v>OFFICIAL</x:v>
-      </x:c>
-      <x:c r="C30" s="30" t="str">
-        <x:v>Национальное управление миграции Аргентины</x:v>
-      </x:c>
-      <x:c r="D30" s="30" t="str">
-        <x:v>Изменение финансового правила рантье и пенсионера 2023 года</x:v>
-      </x:c>
-      <x:c r="E30" s="30" t="str">
-        <x:v>https://www.argentina.gob.ar/normativa/nacional/disposici%C3%B3n-3446-2023-392424/texto</x:v>
-      </x:c>
-      <x:c r="F30" s="30" t="str">
-        <x:v>Действующая формулировка: минимум 5 официальных минимальных зарплат; прежняя фраза о сумме на каждого заявителя заменена.</x:v>
-      </x:c>
-      <x:c r="G30" s="30" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="H30" s="30" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
+      <x:c r="A30" s="30"/>
+      <x:c r="B30" s="30"/>
+      <x:c r="C30" s="30"/>
+      <x:c r="D30" s="30"/>
+      <x:c r="E30" s="30"/>
+      <x:c r="F30" s="30"/>
+      <x:c r="G30" s="30"/>
+      <x:c r="H30" s="30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1690,7 +1688,7 @@
         <x:v>Не разъяснён зачёт краткосрочной резиденции цифрового кочевника в гражданство.</x:v>
       </x:c>
       <x:c r="E4" s="30" t="str">
-        <x:v>Не засчитывать период и показывать необходимость перехода на долгосрочный статус.</x:v>
+        <x:v>Не засчитывать краткосрочный статус в срок гражданства и прямо указывать, что он не соответствует обязательной долгосрочной цели.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1755,6 +1753,16 @@
     <x:row r="7">
       <x:c r="A7" s="26" t="str">
         <x:v>Чип, вакцина, титр антител, перевозка и аренда жилья с животными.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Маршруты, требующие гражданства, отличного от гражданства РФ, включая гражданство страны МЕРКОСУР.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Воссоединение с гражданином или резидентом страны назначения как самостоятельное основание для подбора страны.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1798,7 +1806,7 @@
         <x:v>Маршрутов всего</x:v>
       </x:c>
       <x:c r="B3" s="10" t="n">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>OK</x:v>
@@ -1809,7 +1817,7 @@
         <x:v>Публикуемых маршрутов</x:v>
       </x:c>
       <x:c r="B4" s="10" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
         <x:v>OK</x:v>
@@ -1853,7 +1861,7 @@
         <x:v>Источников</x:v>
       </x:c>
       <x:c r="B8" s="10" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>OK</x:v>
@@ -1872,12 +1880,23 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="str">
+        <x:v>Ожидаемых изменений</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
         <x:v>Общая полнота</x:v>
       </x:c>
-      <x:c r="B10" s="10" t="str">
+      <x:c r="B11" t="str">
         <x:v>92%</x:v>
       </x:c>
-      <x:c r="C10" s="10" t="str">
+      <x:c r="C11" t="str">
         <x:v>REVIEW</x:v>
       </x:c>
     </x:row>
@@ -1929,10 +1948,10 @@
         <x:v>Argentina</x:v>
       </x:c>
       <x:c r="D2" s="30" t="str">
-        <x:v>Для гражданина РФ подтверждены 8 публикуемых маршрутов. Цифровой кочевник доступен благодаря безвизовому туристическому въезду, но является краткосрочным статусом. Долгосрочные основания: пассивный доход, пенсия, местная работа, квалифицированная работа или внутрикорпоративный перевод, учёба, семья и подходящее второе гражданство МЕРКОСУР.</x:v>
+        <x:v>Для гражданина РФ подтверждены 6 маршрутов, которые можно оценить по универсальной анкете: цифровой кочевник, пассивный доход, пенсия, местная работа, квалифицированная работа или внутрикорпоративный перевод и учёба. Цифровой кочевник является краткосрочным статусом.</x:v>
       </x:c>
       <x:c r="E2" s="30" t="str">
-        <x:v>Готова к подключению для 8 маршрутов; инвесторская резиденция и гражданство за инвестицию скрыты до публикации критериев.</x:v>
+        <x:v>Готова к подключению для 6 маршрутов, которые можно оценить по универсальной анкете гражданина РФ; инвесторская резиденция скрыта до публикации критериев.</x:v>
       </x:c>
       <x:c r="F2" s="30" t="n">
         <x:v>92</x:v>
@@ -2229,115 +2248,69 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
-        <x:v>AR_FAMILY</x:v>
+        <x:v>AR_INVESTOR_HIDDEN</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>Временная резиденция по воссоединению семьи</x:v>
+        <x:v>Временная резиденция инвестора</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>reunificación familiar — воссоединение семьи</x:v>
+        <x:v>residencia temporaria como inversionista — временная резиденция инвестора</x:v>
       </x:c>
       <x:c r="D8" s="30" t="str">
-        <x:v>FAMILY_REUNIFICATION</x:v>
+        <x:v>INVESTOR</x:v>
       </x:c>
       <x:c r="E8" s="30" t="str">
-        <x:v>ДА</x:v>
+        <x:v>НЕТ</x:v>
       </x:c>
       <x:c r="F8" s="30" t="str">
-        <x:v>ДА</x:v>
+        <x:v>LEGAL_CATEGORY_EXISTS_BUT_PROCEDURE_NOT_PUBLISHED</x:v>
       </x:c>
       <x:c r="G8" s="30" t="str">
-        <x:v>Признанная семейная связь с гражданином или временным/постоянным резидентом Аргентины.</x:v>
+        <x:v>Внесение собственных активов для деятельности, представляющей интерес для Аргентины.</x:v>
       </x:c>
       <x:c r="H8" s="30" t="str">
-        <x:v>Через RaDEX.</x:v>
+        <x:v>Актуальная рабочая процедура не найдена на публичном портале.</x:v>
       </x:c>
       <x:c r="I8" s="30" t="str">
-        <x:v>Родственник или резидент-спонсор подаёт на разрешение на въезд; после одобрения заявитель получает визу.</x:v>
+        <x:v>Актуальная рабочая процедура не найдена.</x:v>
       </x:c>
       <x:c r="J8" s="30" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="K8" s="30"/>
+      <x:c r="K8" s="30" t="n">
+        <x:v>36</x:v>
+      </x:c>
       <x:c r="L8" s="30" t="str">
-        <x:v>Подходит, когда семейная связь уже существует и признаётся. Отсутствие официального числового порога дохода не понижает статус.</x:v>
+        <x:v>Скрыт. Нельзя присваивать статус без действующих критериев.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="26" t="str">
-        <x:v>AR_MERCOSUR_SECOND_NATIONALITY</x:v>
-      </x:c>
-      <x:c r="B9" s="26" t="str">
-        <x:v>Временная резиденция по подходящему второму гражданству страны МЕРКОСУР или ассоциированной страны</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="str">
-        <x:v>residencia temporaria por nacionalidad MERCOSUR — временная резиденция по гражданству страны МЕРКОСУР</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>SECOND_CITIZENSHIP_MERCOSUR</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
-      <x:c r="F9" s="26" t="str">
-        <x:v>ONLY_WITH_QUALIFYING_SECOND_CITIZENSHIP</x:v>
-      </x:c>
-      <x:c r="G9" s="26" t="str">
-        <x:v>Подходящее второе гражданство; для некоторых натурализованных граждан требуется не менее 5 лет такого гражданства.</x:v>
-      </x:c>
-      <x:c r="H9" s="26" t="str">
-        <x:v>Через RaDEX.</x:v>
-      </x:c>
-      <x:c r="I9" s="26" t="str">
-        <x:v>Через представителя: разрешение на въезд, затем виза в консульстве.</x:v>
-      </x:c>
-      <x:c r="J9" s="26" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="K9" s="26" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="L9" s="26" t="str">
-        <x:v>Показывается только пользователю с подходящим вторым гражданством.</x:v>
-      </x:c>
+      <x:c r="A9" s="26"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
+      <x:c r="E9" s="26"/>
+      <x:c r="F9" s="26"/>
+      <x:c r="G9" s="26"/>
+      <x:c r="H9" s="26"/>
+      <x:c r="I9" s="26"/>
+      <x:c r="J9" s="26"/>
+      <x:c r="K9" s="26"/>
+      <x:c r="L9" s="26"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="30" t="str">
-        <x:v>AR_INVESTOR_HIDDEN</x:v>
-      </x:c>
-      <x:c r="B10" s="30" t="str">
-        <x:v>Временная резиденция инвестора</x:v>
-      </x:c>
-      <x:c r="C10" s="30" t="str">
-        <x:v>residencia temporaria como inversionista — временная резиденция инвестора</x:v>
-      </x:c>
-      <x:c r="D10" s="30" t="str">
-        <x:v>INVESTOR</x:v>
-      </x:c>
-      <x:c r="E10" s="30" t="str">
-        <x:v>НЕТ</x:v>
-      </x:c>
-      <x:c r="F10" s="30" t="str">
-        <x:v>LEGAL_CATEGORY_EXISTS_BUT_PROCEDURE_NOT_PUBLISHED</x:v>
-      </x:c>
-      <x:c r="G10" s="30" t="str">
-        <x:v>Внесение собственных активов для деятельности, представляющей интерес для Аргентины.</x:v>
-      </x:c>
-      <x:c r="H10" s="30" t="str">
-        <x:v>Актуальная рабочая процедура не найдена на публичном портале.</x:v>
-      </x:c>
-      <x:c r="I10" s="30" t="str">
-        <x:v>Актуальная рабочая процедура не найдена.</x:v>
-      </x:c>
-      <x:c r="J10" s="30" t="n">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="K10" s="30" t="n">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="L10" s="30" t="str">
-        <x:v>Скрыт. Нельзя присваивать статус без действующих критериев.</x:v>
-      </x:c>
+      <x:c r="A10" s="30"/>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="30"/>
+      <x:c r="J10" s="30"/>
+      <x:c r="K10" s="30"/>
+      <x:c r="L10" s="30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2540,16 +2513,16 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
-        <x:v>AR_FAMILY</x:v>
+        <x:v>AR_INVESTOR_HIDDEN</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>Временная резиденция по воссоединению семьи</x:v>
+        <x:v>Временная резиденция инвестора</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>Фиксированного числового порога нет. При подаче из-за рубежа спонсор подтверждает фактические доходы за последние 3 месяца.</x:v>
+        <x:v>Категория существует в законе, но актуальный операционный порог и рабочая процедура не опубликованы.</x:v>
       </x:c>
       <x:c r="D8" s="30" t="str">
-        <x:v>NO_NUMERIC_THRESHOLD</x:v>
+        <x:v>UNKNOWN_NOT_PUBLISHED</x:v>
       </x:c>
       <x:c r="E8" s="30"/>
       <x:c r="F8" s="30"/>
@@ -2558,54 +2531,30 @@
         <x:v>ДА</x:v>
       </x:c>
       <x:c r="I8" s="30" t="str">
-        <x:v>Подходит, когда семейная связь уже существует и признаётся. Отсутствие официального числового порога дохода не понижает статус.</x:v>
+        <x:v>Скрыт. Нельзя присваивать статус без действующих критериев.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="26" t="str">
-        <x:v>AR_MERCOSUR_SECOND_NATIONALITY</x:v>
-      </x:c>
-      <x:c r="B9" s="26" t="str">
-        <x:v>Временная резиденция по подходящему второму гражданству страны МЕРКОСУР или ассоциированной страны</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="str">
-        <x:v>Отдельного доходного порога для основания по гражданству нет.</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>NO_NUMERIC_THRESHOLD</x:v>
-      </x:c>
+      <x:c r="A9" s="26"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
       <x:c r="E9" s="26"/>
       <x:c r="F9" s="26"/>
       <x:c r="G9" s="26"/>
-      <x:c r="H9" s="26" t="str">
-        <x:v>НЕТ</x:v>
-      </x:c>
-      <x:c r="I9" s="26" t="str">
-        <x:v>Показывается только пользователю с подходящим вторым гражданством.</x:v>
-      </x:c>
+      <x:c r="H9" s="26"/>
+      <x:c r="I9" s="26"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="30" t="str">
-        <x:v>AR_INVESTOR_HIDDEN</x:v>
-      </x:c>
-      <x:c r="B10" s="30" t="str">
-        <x:v>Временная резиденция инвестора</x:v>
-      </x:c>
-      <x:c r="C10" s="30" t="str">
-        <x:v>Категория существует в законе, но актуальный операционный порог и рабочая процедура не опубликованы.</x:v>
-      </x:c>
-      <x:c r="D10" s="30" t="str">
-        <x:v>UNKNOWN_NOT_PUBLISHED</x:v>
-      </x:c>
+      <x:c r="A10" s="30"/>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
       <x:c r="E10" s="30"/>
       <x:c r="F10" s="30"/>
       <x:c r="G10" s="30"/>
-      <x:c r="H10" s="30" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
-      <x:c r="I10" s="30" t="str">
-        <x:v>Скрыт. Нельзя присваивать статус без действующих критериев.</x:v>
-      </x:c>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2722,45 +2671,29 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
-        <x:v>AR_FAMILY</x:v>
+        <x:v>AR_INVESTOR_HIDDEN</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>Временная резиденция по воссоединению семьи</x:v>
+        <x:v>Временная резиденция инвестора</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>Супруг; зарегистрированное фактическое партнёрство — официально зарегистрированное совместное проживание пары без брака; родитель; не состоящий в браке и не эмансипированный ребёнок младше 18 лет; совершеннолетний ребёнок с инвалидностью. Иностранное зарегистрированное фактическое партнёрство предварительно регистрируется в аргентинском ЗАГСе.</x:v>
+        <x:v>Не подключать до публикации действующей процедуры.</x:v>
       </x:c>
       <x:c r="D8" s="30" t="str">
-        <x:v>Временная семейная резиденция разрешает работать по найму и на себя.</x:v>
+        <x:v>Не оценивается до активации маршрута.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="26" t="str">
-        <x:v>AR_MERCOSUR_SECOND_NATIONALITY</x:v>
-      </x:c>
-      <x:c r="B9" s="26" t="str">
-        <x:v>Временная резиденция по подходящему второму гражданству страны МЕРКОСУР или ассоциированной страны</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="str">
-        <x:v>Члены семьи могут использовать отдельный маршрут воссоединения семьи.</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>Партнёр с временной семейной резиденцией вправе работать.</x:v>
-      </x:c>
+      <x:c r="A9" s="26"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="30" t="str">
-        <x:v>AR_INVESTOR_HIDDEN</x:v>
-      </x:c>
-      <x:c r="B10" s="30" t="str">
-        <x:v>Временная резиденция инвестора</x:v>
-      </x:c>
-      <x:c r="C10" s="30" t="str">
-        <x:v>Не подключать до публикации действующей процедуры.</x:v>
-      </x:c>
-      <x:c r="D10" s="30" t="str">
-        <x:v>Не оценивается до активации маршрута.</x:v>
-      </x:c>
+      <x:c r="A10" s="30"/>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2899,10 +2832,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
-        <x:v>AR_FAMILY</x:v>
+        <x:v>AR_INVESTOR_HIDDEN</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>Временная резиденция по воссоединению семьи</x:v>
+        <x:v>Временная резиденция инвестора</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
         <x:v>ДА</x:v>
@@ -2915,38 +2848,18 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="26" t="str">
-        <x:v>AR_MERCOSUR_SECOND_NATIONALITY</x:v>
-      </x:c>
-      <x:c r="B9" s="26" t="str">
-        <x:v>Временная резиденция по подходящему второму гражданству страны МЕРКОСУР или ассоциированной страны</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
+      <x:c r="A9" s="26"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
+      <x:c r="E9" s="26"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="30" t="str">
-        <x:v>AR_INVESTOR_HIDDEN</x:v>
-      </x:c>
-      <x:c r="B10" s="30" t="str">
-        <x:v>Временная резиденция инвестора</x:v>
-      </x:c>
-      <x:c r="C10" s="30" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
-      <x:c r="D10" s="30" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
-      <x:c r="E10" s="30" t="str">
-        <x:v>ДА</x:v>
-      </x:c>
+      <x:c r="A10" s="30"/>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3107,63 +3020,39 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
-        <x:v>AR_FAMILY</x:v>
+        <x:v>AR_INVESTOR_HIDDEN</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>Временная резиденция по воссоединению семьи</x:v>
+        <x:v>Временная резиденция инвестора</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>Для гражданина РФ — общий путь после 3 лет временной резиденции при присутствии более 50% срока. Для отдельных детей граждан Аргентины есть прямое основание ПМЖ.</x:v>
+        <x:v>Категория временная; потенциально общий путь к ПМЖ составляет 3 года, но маршрут скрыт.</x:v>
       </x:c>
       <x:c r="D8" s="30" t="str">
-        <x:v>Для ПМЖ нужно находиться в Аргентине более 50% срока временной резиденции.</x:v>
+        <x:v>Не оценивается до публикации маршрута.</x:v>
       </x:c>
       <x:c r="E8" s="30" t="str">
-        <x:v>Гражданство после 2 непрерывных лет законного проживания без выездов. Брак сам по себе не отменяет общий срок.</x:v>
+        <x:v>Не смешивать с гражданством за значимую инвестицию: критерии этой отдельной программы тоже не опубликованы.</x:v>
       </x:c>
       <x:c r="F8" s="30" t="str">
-        <x:v>Отказ от гражданства РФ не требуется; гражданство РФ сохраняется.</x:v>
+        <x:v>Общее правило сохранения гражданства РФ применимо, но маршрут не публикуется.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="26" t="str">
-        <x:v>AR_MERCOSUR_SECOND_NATIONALITY</x:v>
-      </x:c>
-      <x:c r="B9" s="26" t="str">
-        <x:v>Временная резиденция по подходящему второму гражданству страны МЕРКОСУР или ассоциированной страны</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="str">
-        <x:v>ПМЖ после 2 лет временной резиденции при присутствии более 50% срока.</x:v>
-      </x:c>
-      <x:c r="D9" s="26" t="str">
-        <x:v>Для ПМЖ нужно находиться в Аргентине более 50% срока временной резиденции.</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="str">
-        <x:v>Гражданство после 2 непрерывных лет законного проживания без выездов.</x:v>
-      </x:c>
-      <x:c r="F9" s="26" t="str">
-        <x:v>Отказ от гражданства РФ не требуется; гражданство РФ сохраняется.</x:v>
-      </x:c>
+      <x:c r="A9" s="26"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
+      <x:c r="E9" s="26"/>
+      <x:c r="F9" s="26"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="30" t="str">
-        <x:v>AR_INVESTOR_HIDDEN</x:v>
-      </x:c>
-      <x:c r="B10" s="30" t="str">
-        <x:v>Временная резиденция инвестора</x:v>
-      </x:c>
-      <x:c r="C10" s="30" t="str">
-        <x:v>Категория временная; потенциально общий путь к ПМЖ составляет 3 года, но маршрут скрыт.</x:v>
-      </x:c>
-      <x:c r="D10" s="30" t="str">
-        <x:v>Не оценивается до публикации маршрута.</x:v>
-      </x:c>
-      <x:c r="E10" s="30" t="str">
-        <x:v>Не смешивать с гражданством за значимую инвестицию: критерии этой отдельной программы тоже не опубликованы.</x:v>
-      </x:c>
-      <x:c r="F10" s="30" t="str">
-        <x:v>Общее правило сохранения гражданства РФ применимо, но маршрут не публикуется.</x:v>
-      </x:c>
+      <x:c r="A10" s="30"/>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3238,7 +3127,7 @@
         <x:v>Буэнос-Айрес</x:v>
       </x:c>
       <x:c r="C2" s="30" t="str">
-        <x:v>["столица", "самый дорогой из выбранных городов"]</x:v>
+        <x:v>["столица", "самый дорогой"]</x:v>
       </x:c>
       <x:c r="D2" s="30" t="str">
         <x:v>крупный</x:v>
@@ -3279,7 +3168,7 @@
         <x:v>Сантьяго-дель-Эстеро</x:v>
       </x:c>
       <x:c r="C3" s="26" t="str">
-        <x:v>["самый недорогой из выбранных городов", "самый жаркий из выбранных городов"]</x:v>
+        <x:v>["самый жаркий"]</x:v>
       </x:c>
       <x:c r="D3" s="26" t="str">
         <x:v>средний</x:v>
@@ -3320,7 +3209,7 @@
         <x:v>Ушуайя</x:v>
       </x:c>
       <x:c r="C4" s="30" t="str">
-        <x:v>["самый холодный из выбранных городов"]</x:v>
+        <x:v>["самый недорогой", "самый холодный"]</x:v>
       </x:c>
       <x:c r="D4" s="30" t="str">
         <x:v>небольшой</x:v>

</xml_diff>